<commit_message>
ENS y mayor y menos a 2 MW
</commit_message>
<xml_diff>
--- a/Mantenimientos planificados CNEL EP 30-31 mayo y 6-7junio version final.xlsx
+++ b/Mantenimientos planificados CNEL EP 30-31 mayo y 6-7junio version final.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\solange.doylet\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.ulloa\Documents\GitHub\dashboard-mantenimientos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12015"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$W$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$J$40</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -1284,22 +1284,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="38"/>
-    <col min="2" max="2" width="50.28515625" style="38" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" style="38" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="38" customWidth="1"/>
-    <col min="5" max="9" width="11.42578125" style="38"/>
-    <col min="10" max="10" width="12.85546875" style="38" customWidth="1"/>
-    <col min="11" max="14" width="11.42578125" style="38"/>
+    <col min="1" max="1" width="11.44140625" style="38"/>
+    <col min="2" max="2" width="50.33203125" style="38" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="38" customWidth="1"/>
+    <col min="5" max="9" width="11.44140625" style="38"/>
+    <col min="10" max="10" width="12.88671875" style="38" customWidth="1"/>
+    <col min="11" max="14" width="11.44140625" style="38"/>
     <col min="15" max="15" width="16" style="38" customWidth="1"/>
-    <col min="16" max="16" width="11.42578125" style="38"/>
-    <col min="17" max="17" width="24.85546875" style="38" customWidth="1"/>
-    <col min="18" max="16384" width="11.42578125" style="38"/>
+    <col min="16" max="16" width="11.44140625" style="38"/>
+    <col min="17" max="17" width="24.88671875" style="38" customWidth="1"/>
+    <col min="18" max="16384" width="11.44140625" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="W1" s="7"/>
     </row>
-    <row r="2" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>22</v>
       </c>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="W2" s="14"/>
     </row>
-    <row r="3" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>22</v>
       </c>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="W3" s="14"/>
     </row>
-    <row r="4" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>35</v>
       </c>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="W4" s="14"/>
     </row>
-    <row r="5" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>35</v>
       </c>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="W5" s="14"/>
     </row>
-    <row r="6" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>35</v>
       </c>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="W6" s="14"/>
     </row>
-    <row r="7" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>35</v>
       </c>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="W7" s="14"/>
     </row>
-    <row r="8" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>35</v>
       </c>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="W8" s="14"/>
     </row>
-    <row r="9" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>56</v>
       </c>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="W9" s="14"/>
     </row>
-    <row r="10" spans="1:23" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="61.2" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>56</v>
       </c>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="W10" s="14"/>
     </row>
-    <row r="11" spans="1:23" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="51" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>56</v>
       </c>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="W11" s="14"/>
     </row>
-    <row r="12" spans="1:23" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="51" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>56</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="101.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="91.8" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>56</v>
       </c>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="W13" s="14"/>
     </row>
-    <row r="14" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="71.400000000000006" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>82</v>
       </c>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="W14" s="14"/>
     </row>
-    <row r="15" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="71.400000000000006" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>82</v>
       </c>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="W15" s="14"/>
     </row>
-    <row r="16" spans="1:23" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="40.799999999999997" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>94</v>
       </c>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="W16" s="14"/>
     </row>
-    <row r="17" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>100</v>
       </c>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="W17" s="14"/>
     </row>
-    <row r="18" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>100</v>
       </c>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="W18" s="14"/>
     </row>
-    <row r="19" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>100</v>
       </c>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="W19" s="14"/>
     </row>
-    <row r="20" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" ht="40.799999999999997" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>113</v>
       </c>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="W20" s="14"/>
     </row>
-    <row r="21" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>113</v>
       </c>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="W21" s="14"/>
     </row>
-    <row r="22" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A22" s="23" t="s">
         <v>22</v>
       </c>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="W22" s="7"/>
     </row>
-    <row r="23" spans="1:23" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="51" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
         <v>35</v>
       </c>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="W23" s="7"/>
     </row>
-    <row r="24" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" ht="40.799999999999997" x14ac:dyDescent="0.3">
       <c r="A24" s="23" t="s">
         <v>35</v>
       </c>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="W24" s="7"/>
     </row>
-    <row r="25" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
         <v>35</v>
       </c>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="W25" s="7"/>
     </row>
-    <row r="26" spans="1:23" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="51" x14ac:dyDescent="0.3">
       <c r="A26" s="23" t="s">
         <v>35</v>
       </c>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="W26" s="7"/>
     </row>
-    <row r="27" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A27" s="23" t="s">
         <v>142</v>
       </c>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="W27" s="7"/>
     </row>
-    <row r="28" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A28" s="23" t="s">
         <v>142</v>
       </c>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="W28" s="7"/>
     </row>
-    <row r="29" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
         <v>56</v>
       </c>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="W29" s="7"/>
     </row>
-    <row r="30" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
         <v>56</v>
       </c>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="W30" s="7"/>
     </row>
-    <row r="31" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" ht="71.400000000000006" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>82</v>
       </c>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="W31" s="7"/>
     </row>
-    <row r="32" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
         <v>94</v>
       </c>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="W32" s="7"/>
     </row>
-    <row r="33" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A33" s="23" t="s">
         <v>100</v>
       </c>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="W33" s="7"/>
     </row>
-    <row r="34" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" ht="40.799999999999997" x14ac:dyDescent="0.3">
       <c r="A34" s="23" t="s">
         <v>100</v>
       </c>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="W34" s="7"/>
     </row>
-    <row r="35" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A35" s="23" t="s">
         <v>113</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="37" spans="1:23" s="49" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:23" s="49" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.2">
       <c r="A37" s="39" t="s">
         <v>94</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A38" s="51" t="s">
         <v>56</v>
       </c>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="W38" s="7"/>
     </row>
-    <row r="39" spans="1:23" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A39" s="51" t="s">
         <v>56</v>
       </c>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="W39" s="7"/>
     </row>
-    <row r="40" spans="1:23" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A40" s="51" t="s">
         <v>56</v>
       </c>
@@ -3876,6 +3876,7 @@
       <c r="W40" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J40"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>